<commit_message>
Updated CHN_grids_kan60 model - 2026-09-28 21:41
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_CHN_grids_kan60/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB74B43B-3161-446C-8549-EF36BD33CE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5BE255-5F25-4374-9357-86637CD2DD66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12772" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -1168,10 +1168,10 @@
         <v>86</v>
       </c>
       <c r="M11" t="s">
-        <v>181</v>
+        <v>114</v>
       </c>
       <c r="N11" t="s">
-        <v>182</v>
+        <v>115</v>
       </c>
       <c r="O11" t="s">
         <v>207</v>
@@ -1230,10 +1230,10 @@
         <v>86</v>
       </c>
       <c r="M12" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
       <c r="N12" t="s">
-        <v>138</v>
+        <v>172</v>
       </c>
       <c r="O12" t="s">
         <v>207</v>
@@ -1292,10 +1292,10 @@
         <v>86</v>
       </c>
       <c r="M13" t="s">
-        <v>104</v>
+        <v>187</v>
       </c>
       <c r="N13" t="s">
-        <v>105</v>
+        <v>188</v>
       </c>
       <c r="O13" t="s">
         <v>207</v>
@@ -1354,10 +1354,10 @@
         <v>86</v>
       </c>
       <c r="M14" t="s">
-        <v>191</v>
+        <v>137</v>
       </c>
       <c r="N14" t="s">
-        <v>192</v>
+        <v>138</v>
       </c>
       <c r="O14" t="s">
         <v>207</v>
@@ -1416,10 +1416,10 @@
         <v>86</v>
       </c>
       <c r="M15" t="s">
-        <v>159</v>
+        <v>179</v>
       </c>
       <c r="N15" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="O15" t="s">
         <v>207</v>
@@ -1478,10 +1478,10 @@
         <v>86</v>
       </c>
       <c r="M16" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="N16" t="s">
-        <v>101</v>
+        <v>127</v>
       </c>
       <c r="O16" t="s">
         <v>207</v>
@@ -1540,10 +1540,10 @@
         <v>86</v>
       </c>
       <c r="M17" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="N17" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="O17" t="s">
         <v>207</v>
@@ -1602,10 +1602,10 @@
         <v>86</v>
       </c>
       <c r="M18" t="s">
-        <v>114</v>
+        <v>199</v>
       </c>
       <c r="N18" t="s">
-        <v>115</v>
+        <v>200</v>
       </c>
       <c r="O18" t="s">
         <v>207</v>
@@ -1664,10 +1664,10 @@
         <v>86</v>
       </c>
       <c r="M19" t="s">
-        <v>179</v>
+        <v>135</v>
       </c>
       <c r="N19" t="s">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="O19" t="s">
         <v>207</v>
@@ -1726,10 +1726,10 @@
         <v>86</v>
       </c>
       <c r="M20" t="s">
-        <v>201</v>
+        <v>104</v>
       </c>
       <c r="N20" t="s">
-        <v>202</v>
+        <v>105</v>
       </c>
       <c r="O20" t="s">
         <v>207</v>
@@ -1788,10 +1788,10 @@
         <v>86</v>
       </c>
       <c r="M21" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="N21" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="O21" t="s">
         <v>207</v>
@@ -1850,10 +1850,10 @@
         <v>86</v>
       </c>
       <c r="M22" t="s">
-        <v>197</v>
+        <v>106</v>
       </c>
       <c r="N22" t="s">
-        <v>198</v>
+        <v>107</v>
       </c>
       <c r="O22" t="s">
         <v>207</v>
@@ -1912,10 +1912,10 @@
         <v>86</v>
       </c>
       <c r="M23" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="N23" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="O23" t="s">
         <v>207</v>
@@ -1974,10 +1974,10 @@
         <v>86</v>
       </c>
       <c r="M24" t="s">
-        <v>118</v>
+        <v>189</v>
       </c>
       <c r="N24" t="s">
-        <v>119</v>
+        <v>190</v>
       </c>
       <c r="O24" t="s">
         <v>207</v>
@@ -2036,10 +2036,10 @@
         <v>86</v>
       </c>
       <c r="M25" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="N25" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="O25" t="s">
         <v>207</v>
@@ -2098,10 +2098,10 @@
         <v>86</v>
       </c>
       <c r="M26" t="s">
-        <v>195</v>
+        <v>100</v>
       </c>
       <c r="N26" t="s">
-        <v>196</v>
+        <v>101</v>
       </c>
       <c r="O26" t="s">
         <v>207</v>
@@ -2160,10 +2160,10 @@
         <v>86</v>
       </c>
       <c r="M27" t="s">
-        <v>120</v>
+        <v>181</v>
       </c>
       <c r="N27" t="s">
-        <v>121</v>
+        <v>182</v>
       </c>
       <c r="O27" t="s">
         <v>207</v>
@@ -2222,10 +2222,10 @@
         <v>86</v>
       </c>
       <c r="M28" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="N28" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="O28" t="s">
         <v>207</v>
@@ -2284,10 +2284,10 @@
         <v>86</v>
       </c>
       <c r="M29" t="s">
-        <v>187</v>
+        <v>122</v>
       </c>
       <c r="N29" t="s">
-        <v>188</v>
+        <v>123</v>
       </c>
       <c r="O29" t="s">
         <v>207</v>
@@ -2346,10 +2346,10 @@
         <v>86</v>
       </c>
       <c r="M30" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="N30" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="O30" t="s">
         <v>207</v>
@@ -2408,10 +2408,10 @@
         <v>86</v>
       </c>
       <c r="M31" t="s">
-        <v>112</v>
+        <v>185</v>
       </c>
       <c r="N31" t="s">
-        <v>113</v>
+        <v>186</v>
       </c>
       <c r="O31" t="s">
         <v>207</v>
@@ -2470,10 +2470,10 @@
         <v>86</v>
       </c>
       <c r="M32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="N32" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O32" t="s">
         <v>207</v>
@@ -2520,10 +2520,10 @@
         <v>86</v>
       </c>
       <c r="M33" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="N33" t="s">
-        <v>125</v>
+        <v>156</v>
       </c>
       <c r="O33" t="s">
         <v>207</v>
@@ -2570,10 +2570,10 @@
         <v>86</v>
       </c>
       <c r="M34" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="N34" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="O34" t="s">
         <v>207</v>
@@ -2620,10 +2620,10 @@
         <v>86</v>
       </c>
       <c r="M35" t="s">
-        <v>98</v>
+        <v>191</v>
       </c>
       <c r="N35" t="s">
-        <v>99</v>
+        <v>192</v>
       </c>
       <c r="O35" t="s">
         <v>207</v>
@@ -2670,10 +2670,10 @@
         <v>86</v>
       </c>
       <c r="M36" t="s">
-        <v>110</v>
+        <v>177</v>
       </c>
       <c r="N36" t="s">
-        <v>111</v>
+        <v>178</v>
       </c>
       <c r="O36" t="s">
         <v>207</v>
@@ -2720,10 +2720,10 @@
         <v>86</v>
       </c>
       <c r="M37" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="N37" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="O37" t="s">
         <v>207</v>
@@ -2770,10 +2770,10 @@
         <v>86</v>
       </c>
       <c r="M38" t="s">
-        <v>205</v>
+        <v>102</v>
       </c>
       <c r="N38" t="s">
-        <v>206</v>
+        <v>103</v>
       </c>
       <c r="O38" t="s">
         <v>207</v>
@@ -2820,10 +2820,10 @@
         <v>86</v>
       </c>
       <c r="M39" t="s">
-        <v>171</v>
+        <v>143</v>
       </c>
       <c r="N39" t="s">
-        <v>172</v>
+        <v>144</v>
       </c>
       <c r="O39" t="s">
         <v>207</v>
@@ -2870,10 +2870,10 @@
         <v>86</v>
       </c>
       <c r="M40" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="N40" t="s">
-        <v>134</v>
+        <v>196</v>
       </c>
       <c r="O40" t="s">
         <v>207</v>
@@ -2920,10 +2920,10 @@
         <v>86</v>
       </c>
       <c r="M41" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="N41" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="O41" t="s">
         <v>207</v>
@@ -2970,10 +2970,10 @@
         <v>86</v>
       </c>
       <c r="M42" t="s">
-        <v>167</v>
+        <v>124</v>
       </c>
       <c r="N42" t="s">
-        <v>168</v>
+        <v>125</v>
       </c>
       <c r="O42" t="s">
         <v>207</v>
@@ -3020,10 +3020,10 @@
         <v>86</v>
       </c>
       <c r="M43" t="s">
-        <v>203</v>
+        <v>173</v>
       </c>
       <c r="N43" t="s">
-        <v>204</v>
+        <v>174</v>
       </c>
       <c r="O43" t="s">
         <v>207</v>
@@ -3070,10 +3070,10 @@
         <v>86</v>
       </c>
       <c r="M44" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="N44" t="s">
-        <v>170</v>
+        <v>204</v>
       </c>
       <c r="O44" t="s">
         <v>207</v>
@@ -3120,10 +3120,10 @@
         <v>86</v>
       </c>
       <c r="M45" t="s">
-        <v>175</v>
+        <v>141</v>
       </c>
       <c r="N45" t="s">
-        <v>176</v>
+        <v>142</v>
       </c>
       <c r="O45" t="s">
         <v>207</v>
@@ -3170,10 +3170,10 @@
         <v>86</v>
       </c>
       <c r="M46" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="N46" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="O46" t="s">
         <v>207</v>
@@ -3220,10 +3220,10 @@
         <v>86</v>
       </c>
       <c r="M47" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N47" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O47" t="s">
         <v>207</v>
@@ -3270,10 +3270,10 @@
         <v>86</v>
       </c>
       <c r="M48" t="s">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="N48" t="s">
-        <v>154</v>
+        <v>206</v>
       </c>
       <c r="O48" t="s">
         <v>207</v>
@@ -3320,10 +3320,10 @@
         <v>86</v>
       </c>
       <c r="M49" t="s">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="N49" t="s">
-        <v>162</v>
+        <v>198</v>
       </c>
       <c r="O49" t="s">
         <v>207</v>
@@ -3370,10 +3370,10 @@
         <v>86</v>
       </c>
       <c r="M50" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="N50" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="O50" t="s">
         <v>207</v>
@@ -3420,10 +3420,10 @@
         <v>86</v>
       </c>
       <c r="M51" t="s">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="N51" t="s">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="O51" t="s">
         <v>207</v>
@@ -3470,10 +3470,10 @@
         <v>86</v>
       </c>
       <c r="M52" t="s">
-        <v>139</v>
+        <v>108</v>
       </c>
       <c r="N52" t="s">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="O52" t="s">
         <v>207</v>
@@ -3520,10 +3520,10 @@
         <v>86</v>
       </c>
       <c r="M53" t="s">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="N53" t="s">
-        <v>107</v>
+        <v>150</v>
       </c>
       <c r="O53" t="s">
         <v>207</v>
@@ -3570,10 +3570,10 @@
         <v>86</v>
       </c>
       <c r="M54" t="s">
-        <v>199</v>
+        <v>92</v>
       </c>
       <c r="N54" t="s">
-        <v>200</v>
+        <v>93</v>
       </c>
       <c r="O54" t="s">
         <v>207</v>
@@ -3620,10 +3620,10 @@
         <v>86</v>
       </c>
       <c r="M55" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="N55" t="s">
-        <v>136</v>
+        <v>166</v>
       </c>
       <c r="O55" t="s">
         <v>207</v>
@@ -3670,10 +3670,10 @@
         <v>86</v>
       </c>
       <c r="M56" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
       <c r="N56" t="s">
-        <v>95</v>
+        <v>152</v>
       </c>
       <c r="O56" t="s">
         <v>207</v>
@@ -3720,10 +3720,10 @@
         <v>86</v>
       </c>
       <c r="M57" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="N57" t="s">
-        <v>166</v>
+        <v>140</v>
       </c>
       <c r="O57" t="s">
         <v>207</v>
@@ -3770,10 +3770,10 @@
         <v>86</v>
       </c>
       <c r="M58" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="N58" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="O58" t="s">
         <v>207</v>
@@ -3820,10 +3820,10 @@
         <v>86</v>
       </c>
       <c r="M59" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="N59" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="O59" t="s">
         <v>207</v>
@@ -3870,10 +3870,10 @@
         <v>86</v>
       </c>
       <c r="M60" t="s">
-        <v>189</v>
+        <v>157</v>
       </c>
       <c r="N60" t="s">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="O60" t="s">
         <v>207</v>
@@ -3920,10 +3920,10 @@
         <v>86</v>
       </c>
       <c r="M61" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="N61" t="s">
-        <v>129</v>
+        <v>88</v>
       </c>
       <c r="O61" t="s">
         <v>207</v>
@@ -3970,10 +3970,10 @@
         <v>86</v>
       </c>
       <c r="M62" t="s">
-        <v>147</v>
+        <v>201</v>
       </c>
       <c r="N62" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="O62" t="s">
         <v>207</v>
@@ -4020,10 +4020,10 @@
         <v>86</v>
       </c>
       <c r="M63" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="N63" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="O63" t="s">
         <v>207</v>
@@ -4070,10 +4070,10 @@
         <v>86</v>
       </c>
       <c r="M64" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="N64" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="O64" t="s">
         <v>207</v>
@@ -4120,10 +4120,10 @@
         <v>86</v>
       </c>
       <c r="M65" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="N65" t="s">
-        <v>156</v>
+        <v>134</v>
       </c>
       <c r="O65" t="s">
         <v>207</v>
@@ -4170,10 +4170,10 @@
         <v>86</v>
       </c>
       <c r="M66" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="N66" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="O66" t="s">
         <v>207</v>
@@ -4220,10 +4220,10 @@
         <v>86</v>
       </c>
       <c r="M67" t="s">
-        <v>193</v>
+        <v>145</v>
       </c>
       <c r="N67" t="s">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="O67" t="s">
         <v>207</v>
@@ -4270,10 +4270,10 @@
         <v>86</v>
       </c>
       <c r="M68" t="s">
-        <v>157</v>
+        <v>96</v>
       </c>
       <c r="N68" t="s">
-        <v>158</v>
+        <v>97</v>
       </c>
       <c r="O68" t="s">
         <v>207</v>
@@ -4320,10 +4320,10 @@
         <v>86</v>
       </c>
       <c r="M69" t="s">
-        <v>177</v>
+        <v>110</v>
       </c>
       <c r="N69" t="s">
-        <v>178</v>
+        <v>111</v>
       </c>
       <c r="O69" t="s">
         <v>207</v>

</xml_diff>

<commit_message>
Updated CHN_grids_kan60 model - 2026-09-30 10:32
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_CHN_grids_kan60/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5BE255-5F25-4374-9357-86637CD2DD66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52B2C74-7DA9-414D-80F1-C7C5B7B52432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12772" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12773" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -1168,10 +1168,10 @@
         <v>86</v>
       </c>
       <c r="M11" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="N11" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="O11" t="s">
         <v>207</v>
@@ -1230,10 +1230,10 @@
         <v>86</v>
       </c>
       <c r="M12" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="N12" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="O12" t="s">
         <v>207</v>
@@ -1292,10 +1292,10 @@
         <v>86</v>
       </c>
       <c r="M13" t="s">
-        <v>187</v>
+        <v>102</v>
       </c>
       <c r="N13" t="s">
-        <v>188</v>
+        <v>103</v>
       </c>
       <c r="O13" t="s">
         <v>207</v>
@@ -1354,10 +1354,10 @@
         <v>86</v>
       </c>
       <c r="M14" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
       <c r="N14" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
       <c r="O14" t="s">
         <v>207</v>
@@ -1416,10 +1416,10 @@
         <v>86</v>
       </c>
       <c r="M15" t="s">
-        <v>179</v>
+        <v>100</v>
       </c>
       <c r="N15" t="s">
-        <v>180</v>
+        <v>101</v>
       </c>
       <c r="O15" t="s">
         <v>207</v>
@@ -1478,10 +1478,10 @@
         <v>86</v>
       </c>
       <c r="M16" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="N16" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="O16" t="s">
         <v>207</v>
@@ -1540,10 +1540,10 @@
         <v>86</v>
       </c>
       <c r="M17" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="N17" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="O17" t="s">
         <v>207</v>
@@ -1602,10 +1602,10 @@
         <v>86</v>
       </c>
       <c r="M18" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="N18" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="O18" t="s">
         <v>207</v>
@@ -1664,10 +1664,10 @@
         <v>86</v>
       </c>
       <c r="M19" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="N19" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="O19" t="s">
         <v>207</v>
@@ -1726,10 +1726,10 @@
         <v>86</v>
       </c>
       <c r="M20" t="s">
-        <v>104</v>
+        <v>181</v>
       </c>
       <c r="N20" t="s">
-        <v>105</v>
+        <v>182</v>
       </c>
       <c r="O20" t="s">
         <v>207</v>
@@ -1788,10 +1788,10 @@
         <v>86</v>
       </c>
       <c r="M21" t="s">
-        <v>167</v>
+        <v>112</v>
       </c>
       <c r="N21" t="s">
-        <v>168</v>
+        <v>113</v>
       </c>
       <c r="O21" t="s">
         <v>207</v>
@@ -1850,10 +1850,10 @@
         <v>86</v>
       </c>
       <c r="M22" t="s">
-        <v>106</v>
+        <v>163</v>
       </c>
       <c r="N22" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="O22" t="s">
         <v>207</v>
@@ -1912,10 +1912,10 @@
         <v>86</v>
       </c>
       <c r="M23" t="s">
-        <v>153</v>
+        <v>98</v>
       </c>
       <c r="N23" t="s">
-        <v>154</v>
+        <v>99</v>
       </c>
       <c r="O23" t="s">
         <v>207</v>
@@ -1974,10 +1974,10 @@
         <v>86</v>
       </c>
       <c r="M24" t="s">
-        <v>189</v>
+        <v>110</v>
       </c>
       <c r="N24" t="s">
-        <v>190</v>
+        <v>111</v>
       </c>
       <c r="O24" t="s">
         <v>207</v>
@@ -2036,10 +2036,10 @@
         <v>86</v>
       </c>
       <c r="M25" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="N25" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="O25" t="s">
         <v>207</v>
@@ -2098,10 +2098,10 @@
         <v>86</v>
       </c>
       <c r="M26" t="s">
-        <v>100</v>
+        <v>183</v>
       </c>
       <c r="N26" t="s">
-        <v>101</v>
+        <v>184</v>
       </c>
       <c r="O26" t="s">
         <v>207</v>
@@ -2160,10 +2160,10 @@
         <v>86</v>
       </c>
       <c r="M27" t="s">
-        <v>181</v>
+        <v>96</v>
       </c>
       <c r="N27" t="s">
-        <v>182</v>
+        <v>97</v>
       </c>
       <c r="O27" t="s">
         <v>207</v>
@@ -2222,10 +2222,10 @@
         <v>86</v>
       </c>
       <c r="M28" t="s">
-        <v>116</v>
+        <v>193</v>
       </c>
       <c r="N28" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="O28" t="s">
         <v>207</v>
@@ -2284,10 +2284,10 @@
         <v>86</v>
       </c>
       <c r="M29" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="N29" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="O29" t="s">
         <v>207</v>
@@ -2346,10 +2346,10 @@
         <v>86</v>
       </c>
       <c r="M30" t="s">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="N30" t="s">
-        <v>121</v>
+        <v>166</v>
       </c>
       <c r="O30" t="s">
         <v>207</v>
@@ -2408,10 +2408,10 @@
         <v>86</v>
       </c>
       <c r="M31" t="s">
-        <v>185</v>
+        <v>118</v>
       </c>
       <c r="N31" t="s">
-        <v>186</v>
+        <v>119</v>
       </c>
       <c r="O31" t="s">
         <v>207</v>
@@ -2470,10 +2470,10 @@
         <v>86</v>
       </c>
       <c r="M32" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
       <c r="N32" t="s">
-        <v>148</v>
+        <v>95</v>
       </c>
       <c r="O32" t="s">
         <v>207</v>
@@ -2520,10 +2520,10 @@
         <v>86</v>
       </c>
       <c r="M33" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="N33" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="O33" t="s">
         <v>207</v>
@@ -2570,10 +2570,10 @@
         <v>86</v>
       </c>
       <c r="M34" t="s">
-        <v>90</v>
+        <v>205</v>
       </c>
       <c r="N34" t="s">
-        <v>91</v>
+        <v>206</v>
       </c>
       <c r="O34" t="s">
         <v>207</v>
@@ -2620,10 +2620,10 @@
         <v>86</v>
       </c>
       <c r="M35" t="s">
-        <v>191</v>
+        <v>104</v>
       </c>
       <c r="N35" t="s">
-        <v>192</v>
+        <v>105</v>
       </c>
       <c r="O35" t="s">
         <v>207</v>
@@ -2670,10 +2670,10 @@
         <v>86</v>
       </c>
       <c r="M36" t="s">
-        <v>177</v>
+        <v>90</v>
       </c>
       <c r="N36" t="s">
-        <v>178</v>
+        <v>91</v>
       </c>
       <c r="O36" t="s">
         <v>207</v>
@@ -2720,10 +2720,10 @@
         <v>86</v>
       </c>
       <c r="M37" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="N37" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="O37" t="s">
         <v>207</v>
@@ -2770,10 +2770,10 @@
         <v>86</v>
       </c>
       <c r="M38" t="s">
-        <v>102</v>
+        <v>149</v>
       </c>
       <c r="N38" t="s">
-        <v>103</v>
+        <v>150</v>
       </c>
       <c r="O38" t="s">
         <v>207</v>
@@ -2820,10 +2820,10 @@
         <v>86</v>
       </c>
       <c r="M39" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="N39" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="O39" t="s">
         <v>207</v>
@@ -2870,10 +2870,10 @@
         <v>86</v>
       </c>
       <c r="M40" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
       <c r="N40" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="O40" t="s">
         <v>207</v>
@@ -2920,10 +2920,10 @@
         <v>86</v>
       </c>
       <c r="M41" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="N41" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="O41" t="s">
         <v>207</v>
@@ -2970,10 +2970,10 @@
         <v>86</v>
       </c>
       <c r="M42" t="s">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="N42" t="s">
-        <v>125</v>
+        <v>93</v>
       </c>
       <c r="O42" t="s">
         <v>207</v>
@@ -3020,10 +3020,10 @@
         <v>86</v>
       </c>
       <c r="M43" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="N43" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="O43" t="s">
         <v>207</v>
@@ -3070,10 +3070,10 @@
         <v>86</v>
       </c>
       <c r="M44" t="s">
-        <v>203</v>
+        <v>155</v>
       </c>
       <c r="N44" t="s">
-        <v>204</v>
+        <v>156</v>
       </c>
       <c r="O44" t="s">
         <v>207</v>
@@ -3120,10 +3120,10 @@
         <v>86</v>
       </c>
       <c r="M45" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="N45" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="O45" t="s">
         <v>207</v>
@@ -3220,10 +3220,10 @@
         <v>86</v>
       </c>
       <c r="M47" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="N47" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="O47" t="s">
         <v>207</v>
@@ -3270,10 +3270,10 @@
         <v>86</v>
       </c>
       <c r="M48" t="s">
-        <v>205</v>
+        <v>114</v>
       </c>
       <c r="N48" t="s">
-        <v>206</v>
+        <v>115</v>
       </c>
       <c r="O48" t="s">
         <v>207</v>
@@ -3320,10 +3320,10 @@
         <v>86</v>
       </c>
       <c r="M49" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="N49" t="s">
-        <v>198</v>
+        <v>158</v>
       </c>
       <c r="O49" t="s">
         <v>207</v>
@@ -3370,10 +3370,10 @@
         <v>86</v>
       </c>
       <c r="M50" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="N50" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="O50" t="s">
         <v>207</v>
@@ -3420,10 +3420,10 @@
         <v>86</v>
       </c>
       <c r="M51" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="N51" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="O51" t="s">
         <v>207</v>
@@ -3470,10 +3470,10 @@
         <v>86</v>
       </c>
       <c r="M52" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="N52" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="O52" t="s">
         <v>207</v>
@@ -3520,10 +3520,10 @@
         <v>86</v>
       </c>
       <c r="M53" t="s">
-        <v>149</v>
+        <v>201</v>
       </c>
       <c r="N53" t="s">
-        <v>150</v>
+        <v>202</v>
       </c>
       <c r="O53" t="s">
         <v>207</v>
@@ -3570,10 +3570,10 @@
         <v>86</v>
       </c>
       <c r="M54" t="s">
-        <v>92</v>
+        <v>137</v>
       </c>
       <c r="N54" t="s">
-        <v>93</v>
+        <v>138</v>
       </c>
       <c r="O54" t="s">
         <v>207</v>
@@ -3620,10 +3620,10 @@
         <v>86</v>
       </c>
       <c r="M55" t="s">
-        <v>165</v>
+        <v>203</v>
       </c>
       <c r="N55" t="s">
-        <v>166</v>
+        <v>204</v>
       </c>
       <c r="O55" t="s">
         <v>207</v>
@@ -3670,10 +3670,10 @@
         <v>86</v>
       </c>
       <c r="M56" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="N56" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="O56" t="s">
         <v>207</v>
@@ -3720,10 +3720,10 @@
         <v>86</v>
       </c>
       <c r="M57" t="s">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="N57" t="s">
-        <v>140</v>
+        <v>186</v>
       </c>
       <c r="O57" t="s">
         <v>207</v>
@@ -3770,10 +3770,10 @@
         <v>86</v>
       </c>
       <c r="M58" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="N58" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="O58" t="s">
         <v>207</v>
@@ -3820,10 +3820,10 @@
         <v>86</v>
       </c>
       <c r="M59" t="s">
-        <v>163</v>
+        <v>120</v>
       </c>
       <c r="N59" t="s">
-        <v>164</v>
+        <v>121</v>
       </c>
       <c r="O59" t="s">
         <v>207</v>
@@ -3870,10 +3870,10 @@
         <v>86</v>
       </c>
       <c r="M60" t="s">
-        <v>157</v>
+        <v>133</v>
       </c>
       <c r="N60" t="s">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="O60" t="s">
         <v>207</v>
@@ -3920,10 +3920,10 @@
         <v>86</v>
       </c>
       <c r="M61" t="s">
-        <v>87</v>
+        <v>195</v>
       </c>
       <c r="N61" t="s">
-        <v>88</v>
+        <v>196</v>
       </c>
       <c r="O61" t="s">
         <v>207</v>
@@ -3970,10 +3970,10 @@
         <v>86</v>
       </c>
       <c r="M62" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="N62" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="O62" t="s">
         <v>207</v>
@@ -4020,10 +4020,10 @@
         <v>86</v>
       </c>
       <c r="M63" t="s">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="N63" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="O63" t="s">
         <v>207</v>
@@ -4070,10 +4070,10 @@
         <v>86</v>
       </c>
       <c r="M64" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="N64" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="O64" t="s">
         <v>207</v>
@@ -4120,10 +4120,10 @@
         <v>86</v>
       </c>
       <c r="M65" t="s">
-        <v>133</v>
+        <v>197</v>
       </c>
       <c r="N65" t="s">
-        <v>134</v>
+        <v>198</v>
       </c>
       <c r="O65" t="s">
         <v>207</v>
@@ -4170,10 +4170,10 @@
         <v>86</v>
       </c>
       <c r="M66" t="s">
-        <v>98</v>
+        <v>179</v>
       </c>
       <c r="N66" t="s">
-        <v>99</v>
+        <v>180</v>
       </c>
       <c r="O66" t="s">
         <v>207</v>
@@ -4220,10 +4220,10 @@
         <v>86</v>
       </c>
       <c r="M67" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="N67" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="O67" t="s">
         <v>207</v>
@@ -4270,10 +4270,10 @@
         <v>86</v>
       </c>
       <c r="M68" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="N68" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="O68" t="s">
         <v>207</v>
@@ -4320,10 +4320,10 @@
         <v>86</v>
       </c>
       <c r="M69" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="N69" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="O69" t="s">
         <v>207</v>

</xml_diff>